<commit_message>
Updated Manual testing excel
</commit_message>
<xml_diff>
--- a/Manual Testing.xlsx
+++ b/Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC68F8CF-43C1-45FE-A075-A13FEE88DF64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F591792D-94CE-469F-8EFF-D48D8949268D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4E900C96-DAF3-4DED-B1E4-FC5CD5930C3D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="81">
   <si>
     <t>Characteristics of Software Manual Testing</t>
   </si>
@@ -343,9 +343,6 @@
     <t>hours</t>
   </si>
   <si>
-    <t>Refernce</t>
-  </si>
-  <si>
     <t>https://www.udemy.com/course/comprehensive-software-testing-bootcamp-beginner-to-expert/learn/lecture/42432996#reviews</t>
   </si>
   <si>
@@ -355,12 +352,6 @@
     <t>Acceptance Testing</t>
   </si>
   <si>
-    <t>10:45 - 1:45</t>
-  </si>
-  <si>
-    <t>Make notes in copy with the help of husband</t>
-  </si>
-  <si>
     <t>https://www.tutorialspoint.com/software_testing_dictionary/manual_testing.htm</t>
   </si>
   <si>
@@ -370,9 +361,6 @@
     <t>I opened shopping site and verify the open page, It is visible successfully</t>
   </si>
   <si>
-    <t>I open item and items not shown sizes.</t>
-  </si>
-  <si>
     <t>I add some items in the cart and proceed to checkout. It shows Register / Login account to proceed on checkout.</t>
   </si>
   <si>
@@ -403,19 +391,40 @@
     <t>list of test Cases for practice the Automation(Scenario mentioned in Sheet3)</t>
   </si>
   <si>
-    <t>04:00-05:30</t>
-  </si>
-  <si>
     <t>Git Hub Login Creation, Git Repository creation  &amp; Git Installation</t>
   </si>
   <si>
     <t>https://github.com/shriyagupta1995/CodingAndTesting</t>
   </si>
   <si>
-    <t xml:space="preserve"> Git Installation</t>
-  </si>
-  <si>
-    <t>05:30-06:00</t>
+    <t>Opened items and sizes are not shown.</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Making notes and doing practical work on eclipse</t>
+  </si>
+  <si>
+    <t>Git clone, Git add, Git commit, Git push command learning and practical</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>1.30 hrs</t>
+  </si>
+  <si>
+    <t>30 mins</t>
+  </si>
+  <si>
+    <t>1 hr</t>
+  </si>
+  <si>
+    <t>3 hrs</t>
+  </si>
+  <si>
+    <t>Added this excel and  java practical work to the highlighted repository</t>
   </si>
 </sst>
 </file>
@@ -446,12 +455,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -482,7 +497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -500,13 +515,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1732,7 +1744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C879B6-FFB7-464E-947D-077E910A053A}">
-  <dimension ref="A3:H74"/>
+  <dimension ref="A3:H72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.54296875" bestFit="1" customWidth="1"/>
@@ -1768,7 +1780,7 @@
         <v>52</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
@@ -1811,8 +1823,8 @@
         <v>47</v>
       </c>
       <c r="G6" s="5"/>
-      <c r="H6" s="11" t="s">
-        <v>59</v>
+      <c r="H6" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -1908,7 +1920,7 @@
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -1924,7 +1936,7 @@
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -1940,7 +1952,7 @@
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -1983,8 +1995,8 @@
         <v>47</v>
       </c>
       <c r="G18" s="5"/>
-      <c r="H18" s="11" t="s">
-        <v>59</v>
+      <c r="H18" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -2014,7 +2026,7 @@
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -2030,7 +2042,7 @@
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -2056,7 +2068,7 @@
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -2072,7 +2084,7 @@
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
@@ -2088,7 +2100,7 @@
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -2104,7 +2116,7 @@
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="6" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -2141,16 +2153,16 @@
         <v>45741</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>47</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -2158,15 +2170,13 @@
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
-      <c r="E30" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F30" s="10" t="s">
+      <c r="E30" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F30" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G30" s="3" t="s">
-        <v>57</v>
-      </c>
+      <c r="G30" s="3"/>
       <c r="H30" s="3"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -2174,8 +2184,8 @@
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
-      <c r="E31" s="9" t="s">
-        <v>56</v>
+      <c r="E31" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -2186,7 +2196,7 @@
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
-      <c r="E32" s="9"/>
+      <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
@@ -2196,40 +2206,52 @@
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
-      <c r="E33" s="9"/>
+      <c r="E33" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="F33" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+        <v>66</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="E34" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
-      <c r="E35" s="9" t="s">
-        <v>72</v>
+      <c r="E35" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>71</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="H35" s="3"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
@@ -2237,24 +2259,18 @@
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F36" s="3"/>
-      <c r="G36" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>75</v>
-      </c>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
@@ -2608,26 +2624,6 @@
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
       <c r="H72" s="3"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A74" s="3"/>
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2831,7 +2827,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
@@ -2839,7 +2835,7 @@
         <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
@@ -2847,7 +2843,7 @@
         <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.35">
@@ -2855,7 +2851,7 @@
         <v>4</v>
       </c>
       <c r="B85" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.35">
@@ -2863,12 +2859,12 @@
         <v>5</v>
       </c>
       <c r="B97" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B98" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.35">
@@ -2876,12 +2872,12 @@
         <v>6</v>
       </c>
       <c r="B142" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B143" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.35">
@@ -2889,7 +2885,7 @@
         <v>7</v>
       </c>
       <c r="B164" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Learnings on 7th April 2026
</commit_message>
<xml_diff>
--- a/Manual Testing.xlsx
+++ b/Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Learning\CodingAndTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC3416BB-72E6-49DA-91E9-A5B4F658CDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D673FF-2868-4B30-AF7E-003FFBBE597F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4E900C96-DAF3-4DED-B1E4-FC5CD5930C3D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="143">
   <si>
     <t>Characteristics of Software Manual Testing</t>
   </si>
@@ -579,6 +579,39 @@
   </si>
   <si>
     <t>Continued theoritical learning for Java Roadmap and Rest API.</t>
+  </si>
+  <si>
+    <t>3rd/Monday</t>
+  </si>
+  <si>
+    <t>Multi-threading</t>
+  </si>
+  <si>
+    <t>Git branch</t>
+  </si>
+  <si>
+    <t>Http status codes in Rest API</t>
+  </si>
+  <si>
+    <t>Functional overview of postman and how to test GET request in postman</t>
+  </si>
+  <si>
+    <t>3rd/Tuesday</t>
+  </si>
+  <si>
+    <t>How to create post request and read the json response in postman.</t>
+  </si>
+  <si>
+    <t>How to create put request and read the json response in postman.</t>
+  </si>
+  <si>
+    <t>Trading domain case study</t>
+  </si>
+  <si>
+    <t>Test cases for trading domain case study</t>
+  </si>
+  <si>
+    <t>Created a sample request in postman</t>
   </si>
 </sst>
 </file>
@@ -630,7 +663,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -653,23 +686,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -691,10 +713,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1927,17 +1945,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C879B6-FFB7-464E-947D-077E910A053A}">
-  <dimension ref="A3:H73"/>
+  <dimension ref="A3:H77"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.08984375" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="112.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.08984375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" style="3" customWidth="1"/>
+    <col min="8" max="8" width="112.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
@@ -1977,7 +1996,6 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -2011,9 +2029,6 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
       <c r="D7" s="6"/>
       <c r="E7" s="3" t="s">
         <v>1</v>
@@ -2025,9 +2040,6 @@
       <c r="H7" s="6"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
       <c r="D8" s="6"/>
       <c r="E8" s="3" t="s">
         <v>41</v>
@@ -2039,9 +2051,6 @@
       <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
       <c r="D9" s="6"/>
       <c r="E9" s="3" t="s">
         <v>2</v>
@@ -2053,9 +2062,6 @@
       <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
       <c r="D10" s="6"/>
       <c r="E10" s="3" t="s">
         <v>3</v>
@@ -2067,9 +2073,6 @@
       <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
       <c r="D11" s="6"/>
       <c r="E11" s="3" t="s">
         <v>4</v>
@@ -2081,19 +2084,12 @@
       <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
       <c r="D12" s="6"/>
-      <c r="E12" s="3"/>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
       <c r="D13" s="6"/>
       <c r="E13" s="3" t="s">
         <v>7</v>
@@ -2107,9 +2103,6 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
       <c r="D14" s="6"/>
       <c r="E14" s="3" t="s">
         <v>8</v>
@@ -2123,9 +2116,6 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
       <c r="D15" s="6"/>
       <c r="E15" s="3" t="s">
         <v>9</v>
@@ -2139,19 +2129,12 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
       <c r="D16" s="6"/>
-      <c r="E16" s="3"/>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -2183,144 +2166,84 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
       <c r="E19" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F19" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
       <c r="E20" s="3" t="s">
         <v>39</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G20" s="3"/>
       <c r="H20" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
       <c r="E21" s="3" t="s">
         <v>40</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G21" s="3"/>
       <c r="H21" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
       <c r="F22" s="5"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
       <c r="E23" s="3" t="s">
         <v>35</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G23" s="3"/>
       <c r="H23" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
       <c r="E24" s="3" t="s">
         <v>36</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G24" s="3"/>
       <c r="H24" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
       <c r="E25" s="3" t="s">
         <v>37</v>
       </c>
       <c r="F25" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G25" s="3"/>
       <c r="H25" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
       <c r="E26" s="3" t="s">
         <v>38</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G26" s="3"/>
       <c r="H26" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
       <c r="F27" s="5"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="3">
@@ -2349,46 +2272,19 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
       <c r="E30" s="3" t="s">
         <v>52</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
       <c r="E31" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
       <c r="E33" s="3" t="s">
         <v>65</v>
       </c>
@@ -2403,10 +2299,6 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
       <c r="E34" s="3" t="s">
         <v>66</v>
       </c>
@@ -2421,10 +2313,6 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
       <c r="E35" s="3" t="s">
         <v>71</v>
       </c>
@@ -2434,29 +2322,11 @@
       <c r="G35" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H35" s="3"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
       <c r="E36" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
@@ -2485,9 +2355,6 @@
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
       <c r="D39" s="8"/>
       <c r="E39" s="3" t="s">
         <v>85</v>
@@ -2503,14 +2370,10 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="12" t="s">
+      <c r="E40" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="3" t="s">
         <v>46</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -2521,10 +2384,6 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
       <c r="E41" s="3" t="s">
         <v>78</v>
       </c>
@@ -2534,17 +2393,6 @@
       <c r="G41" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H41" s="3"/>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
@@ -2568,27 +2416,16 @@
       <c r="G43" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H43" s="3"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="D44" s="3"/>
       <c r="E44" s="3" t="s">
         <v>94</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G44" s="3"/>
-      <c r="H44" s="3"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
       <c r="E45" s="3" t="s">
         <v>95</v>
       </c>
@@ -2598,31 +2435,14 @@
       <c r="G45" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H45" s="3"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
       <c r="E46" s="3" t="s">
         <v>96</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="3"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="3">
@@ -2651,10 +2471,6 @@
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
       <c r="E49" s="3" t="s">
         <v>99</v>
       </c>
@@ -2667,16 +2483,6 @@
       <c r="H49" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="3">
@@ -2705,10 +2511,6 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
       <c r="E52" s="3" t="s">
         <v>103</v>
       </c>
@@ -2723,10 +2525,6 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
       <c r="E53" s="3" t="s">
         <v>105</v>
       </c>
@@ -2739,16 +2537,6 @@
       <c r="H53" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="3">
@@ -2769,68 +2557,42 @@
       <c r="F55" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G55" s="3"/>
       <c r="H55" s="7" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
       <c r="E56" s="3" t="s">
         <v>110</v>
       </c>
       <c r="F56" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G56" s="3"/>
       <c r="H56" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
       <c r="E57" s="3" t="s">
         <v>111</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G57" s="3"/>
       <c r="H57" s="7" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
         <v>112</v>
       </c>
       <c r="F58" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G58" s="3"/>
       <c r="H58" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="3">
@@ -2851,68 +2613,42 @@
       <c r="F60" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G60" s="3"/>
       <c r="H60" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
       <c r="E61" s="3" t="s">
         <v>119</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G61" s="3"/>
       <c r="H61" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
       <c r="E62" s="3" t="s">
         <v>121</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G62" s="3"/>
       <c r="H62" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
       <c r="E63" s="3" t="s">
         <v>123</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G63" s="3"/>
       <c r="H63" s="7" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
     </row>
     <row r="65" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="3">
@@ -2927,108 +2663,143 @@
       <c r="D65" s="8">
         <v>46114</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="E65" s="11" t="s">
         <v>127</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G65" s="3"/>
       <c r="H65" s="7" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="13" t="s">
+      <c r="E66" s="11" t="s">
         <v>129</v>
       </c>
       <c r="F66" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G66" s="3"/>
-      <c r="H66" s="14" t="s">
+      <c r="H66" s="12" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
       <c r="E67" s="3" t="s">
         <v>131</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G67" s="3"/>
-      <c r="H67" s="15" t="s">
+      <c r="H67" s="13" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="3"/>
-    </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="3"/>
-      <c r="H69" s="3"/>
+      <c r="A69" s="3">
+        <v>11</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D69" s="8">
+        <v>46118</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H69" s="13" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A70" s="3"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="3"/>
-      <c r="H70" s="3"/>
+      <c r="E70" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="H70" s="13" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
-      <c r="H71" s="3"/>
+      <c r="E71" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H71" s="13" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A73" s="3"/>
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
+      <c r="E72" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H72" s="13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A74" s="3">
+        <v>12</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D74" s="8">
+        <v>46119</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E75" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E76" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E77" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Learnings on 15th April 2026
</commit_message>
<xml_diff>
--- a/Manual Testing.xlsx
+++ b/Manual Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Learning\CodingAndTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E40B77-46D5-48E3-8033-CCCD3FFDB28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870081BA-C302-4893-BA8B-FBA8D3C8B9FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4E900C96-DAF3-4DED-B1E4-FC5CD5930C3D}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet 1" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="182">
   <si>
     <t>Characteristics of Software Manual Testing</t>
   </si>
@@ -664,6 +665,72 @@
   </si>
   <si>
     <t>https://github.com/shriyagupta1995/CodingAndTesting/blob/main/LearningProject/src/com/javalearning/ExcelIOExample.java</t>
+  </si>
+  <si>
+    <t>13/14-04-2026</t>
+  </si>
+  <si>
+    <t>Onine java course</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zIdg7hkqNE0&amp;list=PLu0W_9lII9agS67Uits0UnJyrYiXhDS6q&amp;index=2</t>
+  </si>
+  <si>
+    <t>I opened site and verify the open page, It is visible successfully</t>
+  </si>
+  <si>
+    <t>It directly shows the email ID and tries to register without filling the mandatory fields.</t>
+  </si>
+  <si>
+    <t>Register with a password like '12345'; it is a weak password, and login depends only on the verification code.</t>
+  </si>
+  <si>
+    <t>I downloaded this app, but it only works on certain mobile brands.</t>
+  </si>
+  <si>
+    <t>The account was created successfully, and a confirmation email was received.</t>
+  </si>
+  <si>
+    <t>I installed it many times. It shows the authentication screen, and when I select the second option, it opens the install page again.</t>
+  </si>
+  <si>
+    <t>I installed it again, and it shows a different mobile brand name.</t>
+  </si>
+  <si>
+    <t>Select the Blog option; it opens another page.</t>
+  </si>
+  <si>
+    <t>On this page, the Home, Blog, Categories, and About options are not working.</t>
+  </si>
+  <si>
+    <t>Enter an invalid email format. It shows an error message, and the form is not submitted.</t>
+  </si>
+  <si>
+    <t>https://imalive.co/login</t>
+  </si>
+  <si>
+    <t>case study (Sheet 4)</t>
+  </si>
+  <si>
+    <t>4th/Monday &amp; Tuesday</t>
+  </si>
+  <si>
+    <t>4th Wednesday</t>
+  </si>
+  <si>
+    <t>list of test Cases for practice the "ImAlive" site.</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=b2VJmyarV3I&amp;list=PLu0W_9lII9agS67Uits0UnJyrYiXhDS6q&amp;index=4</t>
+  </si>
+  <si>
+    <t>Create a pattern code that shows different patterns.</t>
+  </si>
+  <si>
+    <t>Learned Lambda expression &amp; created a demo code</t>
+  </si>
+  <si>
+    <t>Learned Multithreading expression &amp; created a demo code</t>
   </si>
 </sst>
 </file>
@@ -1669,6 +1736,407 @@
         <a:xfrm>
           <a:off x="457200" y="30384750"/>
           <a:ext cx="8439584" cy="3086259"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>25401</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7353300</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4A6274B-5C97-0364-D8FD-CF5717582CE1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="635001" y="831849"/>
+          <a:ext cx="7327899" cy="2705101"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>603251</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7727950</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>95465</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFCB7BC7-B46E-42AE-EA73-4624B401F1D5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="603251" y="4203700"/>
+          <a:ext cx="7734299" cy="4178515"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7758045</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>101232</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{378359AC-7420-8E84-E618-F720FC5DA989}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="607392" y="8834783"/>
+          <a:ext cx="7758044" cy="3414275"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>120650</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7747000</xdr:colOff>
+      <xdr:row>115</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1D363464-7741-B9AD-9072-86559937BEC0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="730250" y="12776200"/>
+          <a:ext cx="7626350" cy="3371850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>119</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7702551</xdr:colOff>
+      <xdr:row>137</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E9A004A1-FFEA-669C-2339-ECA0DAE94032}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609601" y="16757650"/>
+          <a:ext cx="7702550" cy="3479800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>141</xdr:row>
+      <xdr:rowOff>31751</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7778750</xdr:colOff>
+      <xdr:row>167</xdr:row>
+      <xdr:rowOff>107951</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3E0DFBF-3ED7-D66D-6BB5-936986982F1D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="635000" y="20840701"/>
+          <a:ext cx="7753350" cy="4864100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7747000</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4FFFC188-1A70-0F44-70AD-1E183AEA9721}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="647700" y="965200"/>
+          <a:ext cx="7708900" cy="2584450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7607301</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{030E461D-A042-CE18-DCD0-A50A749D9213}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609601" y="4051301"/>
+          <a:ext cx="7607300" cy="1212849"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>171</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>7753350</xdr:colOff>
+      <xdr:row>186</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8EDEAED7-837A-6A06-678A-66B66E4D98DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685800" y="31489650"/>
+          <a:ext cx="7677150" cy="2806700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1997,13 +2465,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C879B6-FFB7-464E-947D-077E910A053A}">
-  <dimension ref="A3:H85"/>
+  <dimension ref="A3:H93"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.54296875" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.08984375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="18.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.36328125" style="3" customWidth="1"/>
     <col min="5" max="5" width="65.08984375" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.6328125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="3" customWidth="1"/>
@@ -2947,6 +3415,90 @@
       </c>
       <c r="H85" s="7" t="s">
         <v>159</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A87" s="3">
+        <v>15</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E88" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H88" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E89" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H90" s="7"/>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A91" s="3">
+        <v>16</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D91" s="8">
+        <v>46127</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="H91" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E92" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H92" s="7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E93" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2973,6 +3525,9 @@
     <hyperlink ref="H82" r:id="rId20" xr:uid="{FAFA4C4D-CED3-4B77-ADAB-5A20166AD9FC}"/>
     <hyperlink ref="H84" r:id="rId21" xr:uid="{1F378E46-7459-4932-97FE-D61036462B2D}"/>
     <hyperlink ref="H85" r:id="rId22" xr:uid="{FED8A10C-587B-4F12-846A-F3EB83625812}"/>
+    <hyperlink ref="H88" r:id="rId23" xr:uid="{A66E0165-E1D9-408F-A4C9-1568D4454787}"/>
+    <hyperlink ref="H91" r:id="rId24" xr:uid="{11E99017-3186-41C3-A4AC-A9F921A5F640}"/>
+    <hyperlink ref="H92" r:id="rId25" xr:uid="{812D1945-B736-42A4-A73B-44F5191140D7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3233,4 +3788,98 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2AB819B-7AB1-49AA-824E-0C7B1493A958}">
+  <dimension ref="A2:B171"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="112.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>3</v>
+      </c>
+      <c r="B21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>4</v>
+      </c>
+      <c r="B32" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>5</v>
+      </c>
+      <c r="B50" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>6</v>
+      </c>
+      <c r="B75" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>7</v>
+      </c>
+      <c r="B97" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>8</v>
+      </c>
+      <c r="B118" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A140">
+        <v>9</v>
+      </c>
+      <c r="B140" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A171">
+        <v>10</v>
+      </c>
+      <c r="B171" t="s">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>